<commit_message>
new feature branch with refactored code
</commit_message>
<xml_diff>
--- a/data/input/TBS Price Change Summary Report - October 13th'25.xlsx
+++ b/data/input/TBS Price Change Summary Report - October 13th'25.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://anheuserbuschinbev-my.sharepoint.com/personal/aaditya_singhal_anheuser-busch_com/Documents/FY25/Personal git repo/RevMan-POC-Crew/revman/data/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="8_{0AA89260-8720-4988-BC56-22AC02704366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5994290E-5439-4D97-BFCA-D56C90A9A1C1}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="8_{0AA89260-8720-4988-BC56-22AC02704366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB769AF2-646B-4148-A094-8C8A4914B2C7}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{6A2125F1-4E47-4331-8639-117622155337}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{6A2125F1-4E47-4331-8639-117622155337}"/>
   </bookViews>
   <sheets>
     <sheet name="Price Change Summary Report" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Price Change Summary Report'!$A$8:$M$190</definedName>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="153">
   <si>
     <t>Price Change Summary Report</t>
   </si>
@@ -505,6 +506,9 @@
   </si>
   <si>
     <t>B/C/TC</t>
+  </si>
+  <si>
+    <t>overall validator crew (overall validation)</t>
   </si>
 </sst>
 </file>
@@ -1065,7 +1069,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F88453A7-FECA-4927-826D-F01BE31EC038}">
-  <sheetPr codeName="Sheet4" filterMode="1">
+  <sheetPr codeName="Sheet4">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M190"/>
@@ -1205,7 +1209,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="15.5" hidden="1">
+    <row r="9" spans="1:13" ht="15.5">
       <c r="A9" s="14">
         <v>1065365</v>
       </c>
@@ -1248,7 +1252,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="15.5" hidden="1">
+    <row r="10" spans="1:13" ht="15.5">
       <c r="A10" s="14">
         <v>1129130</v>
       </c>
@@ -1291,7 +1295,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="15.5" hidden="1">
+    <row r="11" spans="1:13" ht="15.5">
       <c r="A11" s="14">
         <v>2042611</v>
       </c>
@@ -1334,7 +1338,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="15.5" hidden="1">
+    <row r="12" spans="1:13" ht="15.5">
       <c r="A12" s="14">
         <v>3353211</v>
       </c>
@@ -1377,7 +1381,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="15.5" hidden="1">
+    <row r="13" spans="1:13" ht="15.5">
       <c r="A13" s="14">
         <v>2503211</v>
       </c>
@@ -1420,7 +1424,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="15.5" hidden="1">
+    <row r="14" spans="1:13" ht="15.5">
       <c r="A14" s="14">
         <v>1143013</v>
       </c>
@@ -1463,7 +1467,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="15.5" hidden="1">
+    <row r="15" spans="1:13" ht="15.5">
       <c r="A15" s="14">
         <v>3891013</v>
       </c>
@@ -1506,7 +1510,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="15.5" hidden="1">
+    <row r="16" spans="1:13" ht="15.5">
       <c r="A16" s="14">
         <v>1617224</v>
       </c>
@@ -1549,7 +1553,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="15.5" hidden="1">
+    <row r="17" spans="1:13" ht="15.5">
       <c r="A17" s="14">
         <v>1035172</v>
       </c>
@@ -1592,7 +1596,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="15.5" hidden="1">
+    <row r="18" spans="1:13" ht="15.5">
       <c r="A18" s="14">
         <v>3891013</v>
       </c>
@@ -1635,7 +1639,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="15.5" hidden="1">
+    <row r="19" spans="1:13" ht="15.5">
       <c r="A19" s="14">
         <v>1465033</v>
       </c>
@@ -1678,7 +1682,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="15.5" hidden="1">
+    <row r="20" spans="1:13" ht="15.5">
       <c r="A20" s="14">
         <v>3583348</v>
       </c>
@@ -1721,7 +1725,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="15.5" hidden="1">
+    <row r="21" spans="1:13" ht="15.5">
       <c r="A21" s="14">
         <v>3582348</v>
       </c>
@@ -1764,7 +1768,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="15.5" hidden="1">
+    <row r="22" spans="1:13" ht="15.5">
       <c r="A22" s="14">
         <v>1504172</v>
       </c>
@@ -1807,7 +1811,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="15.5" hidden="1">
+    <row r="23" spans="1:13" ht="15.5">
       <c r="A23" s="14">
         <v>2341172</v>
       </c>
@@ -1850,7 +1854,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="15.5" hidden="1">
+    <row r="24" spans="1:13" ht="15.5">
       <c r="A24" s="14">
         <v>3353033</v>
       </c>
@@ -1893,7 +1897,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="15.5" hidden="1">
+    <row r="25" spans="1:13" ht="15.5">
       <c r="A25" s="14">
         <v>3879042</v>
       </c>
@@ -1936,7 +1940,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="15.5" hidden="1">
+    <row r="26" spans="1:13" ht="15.5">
       <c r="A26" s="14">
         <v>3154042</v>
       </c>
@@ -1979,7 +1983,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="15.5" hidden="1">
+    <row r="27" spans="1:13" ht="15.5">
       <c r="A27" s="14">
         <v>3715042</v>
       </c>
@@ -2022,7 +2026,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="15.5" hidden="1">
+    <row r="28" spans="1:13" ht="15.5">
       <c r="A28" s="14">
         <v>1090033</v>
       </c>
@@ -2065,7 +2069,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="15.5" hidden="1">
+    <row r="29" spans="1:13" ht="15.5">
       <c r="A29" s="14">
         <v>1060100</v>
       </c>
@@ -2108,7 +2112,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="15.5" hidden="1">
+    <row r="30" spans="1:13" ht="15.5">
       <c r="A30" s="14">
         <v>1879055</v>
       </c>
@@ -2151,7 +2155,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="15.5" hidden="1">
+    <row r="31" spans="1:13" ht="15.5">
       <c r="A31" s="14">
         <v>1873005</v>
       </c>
@@ -2194,7 +2198,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="32" spans="1:13" ht="15.5" hidden="1">
+    <row r="32" spans="1:13" ht="15.5">
       <c r="A32" s="14">
         <v>1599033</v>
       </c>
@@ -2237,7 +2241,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="33" spans="1:13" ht="15.5" hidden="1">
+    <row r="33" spans="1:13" ht="15.5">
       <c r="A33" s="14">
         <v>1584041</v>
       </c>
@@ -2280,7 +2284,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="34" spans="1:13" ht="15.5" hidden="1">
+    <row r="34" spans="1:13" ht="15.5">
       <c r="A34" s="14">
         <v>1584041</v>
       </c>
@@ -2323,7 +2327,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="35" spans="1:13" ht="15.5" hidden="1">
+    <row r="35" spans="1:13" ht="15.5">
       <c r="A35" s="14">
         <v>2022041</v>
       </c>
@@ -2366,7 +2370,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="36" spans="1:13" ht="15.5" hidden="1">
+    <row r="36" spans="1:13" ht="15.5">
       <c r="A36" s="14">
         <v>2022041</v>
       </c>
@@ -2409,7 +2413,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="37" spans="1:13" ht="15.5" hidden="1">
+    <row r="37" spans="1:13" ht="15.5">
       <c r="A37" s="14">
         <v>1065356</v>
       </c>
@@ -2452,7 +2456,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="15.5" hidden="1">
+    <row r="38" spans="1:13" ht="15.5">
       <c r="A38" s="14">
         <v>1448041</v>
       </c>
@@ -2495,7 +2499,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="39" spans="1:13" ht="15.5" hidden="1">
+    <row r="39" spans="1:13" ht="15.5">
       <c r="A39" s="14">
         <v>2042051</v>
       </c>
@@ -2538,7 +2542,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="40" spans="1:13" ht="15.5" hidden="1">
+    <row r="40" spans="1:13" ht="15.5">
       <c r="A40" s="14">
         <v>1319055</v>
       </c>
@@ -2581,7 +2585,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="41" spans="1:13" ht="15.5" hidden="1">
+    <row r="41" spans="1:13" ht="15.5">
       <c r="A41" s="14">
         <v>1045172</v>
       </c>
@@ -2624,7 +2628,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="42" spans="1:13" ht="15.5" hidden="1">
+    <row r="42" spans="1:13" ht="15.5">
       <c r="A42" s="14">
         <v>1026100</v>
       </c>
@@ -2667,7 +2671,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="43" spans="1:13" ht="15.5" hidden="1">
+    <row r="43" spans="1:13" ht="15.5">
       <c r="A43" s="14">
         <v>1030172</v>
       </c>
@@ -2710,7 +2714,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="44" spans="1:13" ht="15.5" hidden="1">
+    <row r="44" spans="1:13" ht="15.5">
       <c r="A44" s="14">
         <v>1056172</v>
       </c>
@@ -2753,7 +2757,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="45" spans="1:13" ht="15.5" hidden="1">
+    <row r="45" spans="1:13" ht="15.5">
       <c r="A45" s="14">
         <v>1628172</v>
       </c>
@@ -2796,7 +2800,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="46" spans="1:13" ht="15.5" hidden="1">
+    <row r="46" spans="1:13" ht="15.5">
       <c r="A46" s="14">
         <v>1490005</v>
       </c>
@@ -2839,7 +2843,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="47" spans="1:13" ht="15.5" hidden="1">
+    <row r="47" spans="1:13" ht="15.5">
       <c r="A47" s="14">
         <v>3353031</v>
       </c>
@@ -2882,7 +2886,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="48" spans="1:13" ht="15.5" hidden="1">
+    <row r="48" spans="1:13" ht="15.5">
       <c r="A48" s="14">
         <v>3888033</v>
       </c>
@@ -2925,7 +2929,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="49" spans="1:13" ht="15.5" hidden="1">
+    <row r="49" spans="1:13" ht="15.5">
       <c r="A49" s="14">
         <v>1041042</v>
       </c>
@@ -2968,7 +2972,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="50" spans="1:13" ht="15.5" hidden="1">
+    <row r="50" spans="1:13" ht="15.5">
       <c r="A50" s="14">
         <v>2598042</v>
       </c>
@@ -3011,7 +3015,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="51" spans="1:13" ht="15.5" hidden="1">
+    <row r="51" spans="1:13" ht="15.5">
       <c r="A51" s="14">
         <v>3666031</v>
       </c>
@@ -3054,7 +3058,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="52" spans="1:13" ht="15.5" hidden="1">
+    <row r="52" spans="1:13" ht="15.5">
       <c r="A52" s="14">
         <v>3654427</v>
       </c>
@@ -3097,7 +3101,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="53" spans="1:13" ht="15.5" hidden="1">
+    <row r="53" spans="1:13" ht="15.5">
       <c r="A53" s="14">
         <v>1056042</v>
       </c>
@@ -3140,7 +3144,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="54" spans="1:13" ht="15.5" hidden="1">
+    <row r="54" spans="1:13" ht="15.5">
       <c r="A54" s="14">
         <v>3668427</v>
       </c>
@@ -3183,7 +3187,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="55" spans="1:13" ht="15.5" hidden="1">
+    <row r="55" spans="1:13" ht="15.5">
       <c r="A55" s="14">
         <v>1595031</v>
       </c>
@@ -3226,7 +3230,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="56" spans="1:13" ht="15.5" hidden="1">
+    <row r="56" spans="1:13" ht="15.5">
       <c r="A56" s="14">
         <v>1594031</v>
       </c>
@@ -3269,7 +3273,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="57" spans="1:13" ht="15.5" hidden="1">
+    <row r="57" spans="1:13" ht="15.5">
       <c r="A57" s="14">
         <v>3962031</v>
       </c>
@@ -3312,7 +3316,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="58" spans="1:13" ht="15.5" hidden="1">
+    <row r="58" spans="1:13" ht="15.5">
       <c r="A58" s="14">
         <v>1491223</v>
       </c>
@@ -3355,7 +3359,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="59" spans="1:13" ht="15.5" hidden="1">
+    <row r="59" spans="1:13" ht="15.5">
       <c r="A59" s="14">
         <v>1491042</v>
       </c>
@@ -3398,7 +3402,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="60" spans="1:13" ht="15.5" hidden="1">
+    <row r="60" spans="1:13" ht="15.5">
       <c r="A60" s="14">
         <v>3410031</v>
       </c>
@@ -3441,7 +3445,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="61" spans="1:13" ht="15.5" hidden="1">
+    <row r="61" spans="1:13" ht="15.5">
       <c r="A61" s="14">
         <v>2042291</v>
       </c>
@@ -3484,7 +3488,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="62" spans="1:13" ht="15.5" hidden="1">
+    <row r="62" spans="1:13" ht="15.5">
       <c r="A62" s="14">
         <v>1056041</v>
       </c>
@@ -3527,7 +3531,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="63" spans="1:13" ht="15.5" hidden="1">
+    <row r="63" spans="1:13" ht="15.5">
       <c r="A63" s="14">
         <v>1491041</v>
       </c>
@@ -3570,7 +3574,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="64" spans="1:13" ht="15.5" hidden="1">
+    <row r="64" spans="1:13" ht="15.5">
       <c r="A64" s="14">
         <v>1525038</v>
       </c>
@@ -3613,7 +3617,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="65" spans="1:13" ht="15.5" hidden="1">
+    <row r="65" spans="1:13" ht="15.5">
       <c r="A65" s="14">
         <v>3879038</v>
       </c>
@@ -3656,7 +3660,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="66" spans="1:13" ht="15.5" hidden="1">
+    <row r="66" spans="1:13" ht="15.5">
       <c r="A66" s="14">
         <v>3154038</v>
       </c>
@@ -3699,7 +3703,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="67" spans="1:13" ht="15.5" hidden="1">
+    <row r="67" spans="1:13" ht="15.5">
       <c r="A67" s="14">
         <v>3715038</v>
       </c>
@@ -3742,7 +3746,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="68" spans="1:13" ht="15.5" hidden="1">
+    <row r="68" spans="1:13" ht="15.5">
       <c r="A68" s="14">
         <v>3775038</v>
       </c>
@@ -3785,7 +3789,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="69" spans="1:13" ht="15.5" hidden="1">
+    <row r="69" spans="1:13" ht="15.5">
       <c r="A69" s="14">
         <v>1628031</v>
       </c>
@@ -3828,7 +3832,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="70" spans="1:13" ht="15.5" hidden="1">
+    <row r="70" spans="1:13" ht="15.5">
       <c r="A70" s="14">
         <v>1491038</v>
       </c>
@@ -3871,7 +3875,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="71" spans="1:13" ht="15.5" hidden="1">
+    <row r="71" spans="1:13" ht="15.5">
       <c r="A71" s="14">
         <v>1448038</v>
       </c>
@@ -3914,7 +3918,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="72" spans="1:13" ht="15.5" hidden="1">
+    <row r="72" spans="1:13" ht="15.5">
       <c r="A72" s="14">
         <v>2042290</v>
       </c>
@@ -3957,7 +3961,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="73" spans="1:13" ht="15.5" hidden="1">
+    <row r="73" spans="1:13" ht="15.5">
       <c r="A73" s="14">
         <v>3537296</v>
       </c>
@@ -4000,7 +4004,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="74" spans="1:13" ht="15.5" hidden="1">
+    <row r="74" spans="1:13" ht="15.5">
       <c r="A74" s="14">
         <v>2042024</v>
       </c>
@@ -4043,7 +4047,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="75" spans="1:13" ht="15.5" hidden="1">
+    <row r="75" spans="1:13" ht="15.5">
       <c r="A75" s="14">
         <v>2084100</v>
       </c>
@@ -4086,7 +4090,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="76" spans="1:13" ht="15.5" hidden="1">
+    <row r="76" spans="1:13" ht="15.5">
       <c r="A76" s="14">
         <v>2085100</v>
       </c>
@@ -4129,7 +4133,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="77" spans="1:13" ht="15.5" hidden="1">
+    <row r="77" spans="1:13" ht="15.5">
       <c r="A77" s="14">
         <v>2597355</v>
       </c>
@@ -4172,7 +4176,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="78" spans="1:13" ht="15.5" hidden="1">
+    <row r="78" spans="1:13" ht="15.5">
       <c r="A78" s="14">
         <v>1629042</v>
       </c>
@@ -4215,7 +4219,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="79" spans="1:13" ht="15.5" hidden="1">
+    <row r="79" spans="1:13" ht="15.5">
       <c r="A79" s="14">
         <v>1628042</v>
       </c>
@@ -4258,7 +4262,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="80" spans="1:13" ht="15.5" hidden="1">
+    <row r="80" spans="1:13" ht="15.5">
       <c r="A80" s="14">
         <v>1041031</v>
       </c>
@@ -4301,7 +4305,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="81" spans="1:13" ht="15.5" hidden="1">
+    <row r="81" spans="1:13" ht="15.5">
       <c r="A81" s="14">
         <v>1035031</v>
       </c>
@@ -4344,7 +4348,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="82" spans="1:13" ht="15.5" hidden="1">
+    <row r="82" spans="1:13" ht="15.5">
       <c r="A82" s="14">
         <v>2598012</v>
       </c>
@@ -4387,7 +4391,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="83" spans="1:13" ht="15.5" hidden="1">
+    <row r="83" spans="1:13" ht="15.5">
       <c r="A83" s="14">
         <v>1448004</v>
       </c>
@@ -4430,7 +4434,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="84" spans="1:13" ht="15.5" hidden="1">
+    <row r="84" spans="1:13" ht="15.5">
       <c r="A84" s="14">
         <v>1119063</v>
       </c>
@@ -4473,7 +4477,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="85" spans="1:13" ht="15.5" hidden="1">
+    <row r="85" spans="1:13" ht="15.5">
       <c r="A85" s="14">
         <v>2662063</v>
       </c>
@@ -4516,7 +4520,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="86" spans="1:13" ht="15.5" hidden="1">
+    <row r="86" spans="1:13" ht="15.5">
       <c r="A86" s="14">
         <v>1161063</v>
       </c>
@@ -4559,7 +4563,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="87" spans="1:13" ht="15.5" hidden="1">
+    <row r="87" spans="1:13" ht="15.5">
       <c r="A87" s="14">
         <v>1632038</v>
       </c>
@@ -4602,7 +4606,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="88" spans="1:13" ht="15.5" hidden="1">
+    <row r="88" spans="1:13" ht="15.5">
       <c r="A88" s="14">
         <v>1629038</v>
       </c>
@@ -4645,7 +4649,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="89" spans="1:13" ht="15.5" hidden="1">
+    <row r="89" spans="1:13" ht="15.5">
       <c r="A89" s="14">
         <v>1628038</v>
       </c>
@@ -4688,7 +4692,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="90" spans="1:13" ht="15.5" hidden="1">
+    <row r="90" spans="1:13" ht="15.5">
       <c r="A90" s="14">
         <v>1219063</v>
       </c>
@@ -4731,7 +4735,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="91" spans="1:13" ht="15.5" hidden="1">
+    <row r="91" spans="1:13" ht="15.5">
       <c r="A91" s="14">
         <v>3452004</v>
       </c>
@@ -4774,7 +4778,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="92" spans="1:13" ht="15.5" hidden="1">
+    <row r="92" spans="1:13" ht="15.5">
       <c r="A92" s="14">
         <v>1620004</v>
       </c>
@@ -4817,7 +4821,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="93" spans="1:13" ht="15.5" hidden="1">
+    <row r="93" spans="1:13" ht="15.5">
       <c r="A93" s="14">
         <v>1194063</v>
       </c>
@@ -4860,7 +4864,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="94" spans="1:13" ht="15.5" hidden="1">
+    <row r="94" spans="1:13" ht="15.5">
       <c r="A94" s="14">
         <v>3154004</v>
       </c>
@@ -4903,7 +4907,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="95" spans="1:13" ht="15.5" hidden="1">
+    <row r="95" spans="1:13" ht="15.5">
       <c r="A95" s="14">
         <v>1624004</v>
       </c>
@@ -4946,7 +4950,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="96" spans="1:13" ht="15.5" hidden="1">
+    <row r="96" spans="1:13" ht="15.5">
       <c r="A96" s="14">
         <v>2975004</v>
       </c>
@@ -4989,7 +4993,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="97" spans="1:13" ht="15.5" hidden="1">
+    <row r="97" spans="1:13" ht="15.5">
       <c r="A97" s="14">
         <v>3715004</v>
       </c>
@@ -5032,7 +5036,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="98" spans="1:13" ht="15.5" hidden="1">
+    <row r="98" spans="1:13" ht="15.5">
       <c r="A98" s="14">
         <v>1584004</v>
       </c>
@@ -5075,7 +5079,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="99" spans="1:13" ht="15.5" hidden="1">
+    <row r="99" spans="1:13" ht="15.5">
       <c r="A99" s="14">
         <v>1584004</v>
       </c>
@@ -5118,7 +5122,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="100" spans="1:13" ht="15.5" hidden="1">
+    <row r="100" spans="1:13" ht="15.5">
       <c r="A100" s="14">
         <v>1617173</v>
       </c>
@@ -5161,7 +5165,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="101" spans="1:13" ht="15.5" hidden="1">
+    <row r="101" spans="1:13" ht="15.5">
       <c r="A101" s="14">
         <v>1631173</v>
       </c>
@@ -5204,7 +5208,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="102" spans="1:13" ht="15.5" hidden="1">
+    <row r="102" spans="1:13" ht="15.5">
       <c r="A102" s="14">
         <v>1065002</v>
       </c>
@@ -5247,7 +5251,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="103" spans="1:13" ht="15.5" hidden="1">
+    <row r="103" spans="1:13" ht="15.5">
       <c r="A103" s="14">
         <v>1709306</v>
       </c>
@@ -5290,7 +5294,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="104" spans="1:13" ht="15.5" hidden="1">
+    <row r="104" spans="1:13" ht="15.5">
       <c r="A104" s="14">
         <v>1065306</v>
       </c>
@@ -5333,7 +5337,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="105" spans="1:13" ht="15.5" hidden="1">
+    <row r="105" spans="1:13" ht="15.5">
       <c r="A105" s="14">
         <v>1208130</v>
       </c>
@@ -5376,7 +5380,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="106" spans="1:13" ht="15.5" hidden="1">
+    <row r="106" spans="1:13" ht="15.5">
       <c r="A106" s="14">
         <v>1617172</v>
       </c>
@@ -5419,7 +5423,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="107" spans="1:13" ht="15.5" hidden="1">
+    <row r="107" spans="1:13" ht="15.5">
       <c r="A107" s="14">
         <v>3878038</v>
       </c>
@@ -5462,7 +5466,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="108" spans="1:13" ht="15.5" hidden="1">
+    <row r="108" spans="1:13" ht="15.5">
       <c r="A108" s="14">
         <v>3718038</v>
       </c>
@@ -5505,7 +5509,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="109" spans="1:13" ht="15.5" hidden="1">
+    <row r="109" spans="1:13" ht="15.5">
       <c r="A109" s="14">
         <v>2662128</v>
       </c>
@@ -5548,7 +5552,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="110" spans="1:13" ht="15.5" hidden="1">
+    <row r="110" spans="1:13" ht="15.5">
       <c r="A110" s="14">
         <v>3261128</v>
       </c>
@@ -5591,7 +5595,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="111" spans="1:13" ht="15.5" hidden="1">
+    <row r="111" spans="1:13" ht="15.5">
       <c r="A111" s="14">
         <v>1161128</v>
       </c>
@@ -5634,7 +5638,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="112" spans="1:13" ht="15.5" hidden="1">
+    <row r="112" spans="1:13" ht="15.5">
       <c r="A112" s="14">
         <v>1497038</v>
       </c>
@@ -5677,7 +5681,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="113" spans="1:13" ht="15.5" hidden="1">
+    <row r="113" spans="1:13" ht="15.5">
       <c r="A113" s="14">
         <v>3849030</v>
       </c>
@@ -5720,7 +5724,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="114" spans="1:13" ht="15.5" hidden="1">
+    <row r="114" spans="1:13" ht="15.5">
       <c r="A114" s="14">
         <v>1065033</v>
       </c>
@@ -5763,7 +5767,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="115" spans="1:13" ht="15.5" hidden="1">
+    <row r="115" spans="1:13" ht="15.5">
       <c r="A115" s="14">
         <v>1167128</v>
       </c>
@@ -5806,7 +5810,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="116" spans="1:13" ht="15.5" hidden="1">
+    <row r="116" spans="1:13" ht="15.5">
       <c r="A116" s="14">
         <v>1497041</v>
       </c>
@@ -5849,7 +5853,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="117" spans="1:13" ht="15.5" hidden="1">
+    <row r="117" spans="1:13" ht="15.5">
       <c r="A117" s="14">
         <v>1060041</v>
       </c>
@@ -5892,7 +5896,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="118" spans="1:13" ht="15.5" hidden="1">
+    <row r="118" spans="1:13" ht="15.5">
       <c r="A118" s="14">
         <v>1595038</v>
       </c>
@@ -5935,7 +5939,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="119" spans="1:13" ht="15.5" hidden="1">
+    <row r="119" spans="1:13" ht="15.5">
       <c r="A119" s="14">
         <v>1416038</v>
       </c>
@@ -5978,7 +5982,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="120" spans="1:13" ht="15.5" hidden="1">
+    <row r="120" spans="1:13" ht="15.5">
       <c r="A120" s="14">
         <v>1425038</v>
       </c>
@@ -6021,7 +6025,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="121" spans="1:13" ht="15.5" hidden="1">
+    <row r="121" spans="1:13" ht="15.5">
       <c r="A121" s="14">
         <v>1035042</v>
       </c>
@@ -6064,7 +6068,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="122" spans="1:13" ht="15.5" hidden="1">
+    <row r="122" spans="1:13" ht="15.5">
       <c r="A122" s="14">
         <v>2597354</v>
       </c>
@@ -6107,7 +6111,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="123" spans="1:13" ht="15.5" hidden="1">
+    <row r="123" spans="1:13" ht="15.5">
       <c r="A123" s="14">
         <v>1497042</v>
       </c>
@@ -6150,7 +6154,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="124" spans="1:13" ht="15.5" hidden="1">
+    <row r="124" spans="1:13" ht="15.5">
       <c r="A124" s="14">
         <v>3879156</v>
       </c>
@@ -6193,7 +6197,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="125" spans="1:13" ht="15.5" hidden="1">
+    <row r="125" spans="1:13" ht="15.5">
       <c r="A125" s="14">
         <v>3154156</v>
       </c>
@@ -6236,7 +6240,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="126" spans="1:13" ht="15.5" hidden="1">
+    <row r="126" spans="1:13" ht="15.5">
       <c r="A126" s="14">
         <v>3715156</v>
       </c>
@@ -6279,7 +6283,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="127" spans="1:13" ht="15.5" hidden="1">
+    <row r="127" spans="1:13" ht="15.5">
       <c r="A127" s="14">
         <v>3916042</v>
       </c>
@@ -6365,7 +6369,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="129" spans="1:13" ht="15.5" hidden="1">
+    <row r="129" spans="1:13" ht="15.5">
       <c r="A129" s="14">
         <v>3915042</v>
       </c>
@@ -6408,7 +6412,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="130" spans="1:13" ht="15.5" hidden="1">
+    <row r="130" spans="1:13" ht="15.5">
       <c r="A130" s="14">
         <v>3168031</v>
       </c>
@@ -6451,7 +6455,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="131" spans="1:13" ht="15.5" hidden="1">
+    <row r="131" spans="1:13" ht="15.5">
       <c r="A131" s="14">
         <v>1060042</v>
       </c>
@@ -6494,7 +6498,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="132" spans="1:13" ht="15.5" hidden="1">
+    <row r="132" spans="1:13" ht="15.5">
       <c r="A132" s="14">
         <v>2341042</v>
       </c>
@@ -6537,7 +6541,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="133" spans="1:13" ht="15.5" hidden="1">
+    <row r="133" spans="1:13" ht="15.5">
       <c r="A133" s="14">
         <v>3867427</v>
       </c>
@@ -6580,7 +6584,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="134" spans="1:13" ht="15.5" hidden="1">
+    <row r="134" spans="1:13" ht="15.5">
       <c r="A134" s="14">
         <v>1465042</v>
       </c>
@@ -6623,7 +6627,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="135" spans="1:13" ht="15.5" hidden="1">
+    <row r="135" spans="1:13" ht="15.5">
       <c r="A135" s="14">
         <v>3870427</v>
       </c>
@@ -6666,7 +6670,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="136" spans="1:13" ht="15.5" hidden="1">
+    <row r="136" spans="1:13" ht="15.5">
       <c r="A136" s="14">
         <v>3866427</v>
       </c>
@@ -6709,7 +6713,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="137" spans="1:13" ht="15.5" hidden="1">
+    <row r="137" spans="1:13" ht="15.5">
       <c r="A137" s="14">
         <v>1628224</v>
       </c>
@@ -6752,7 +6756,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="138" spans="1:13" ht="15.5" hidden="1">
+    <row r="138" spans="1:13" ht="15.5">
       <c r="A138" s="14">
         <v>3839028</v>
       </c>
@@ -6795,7 +6799,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="139" spans="1:13" ht="15.5" hidden="1">
+    <row r="139" spans="1:13" ht="15.5">
       <c r="A139" s="14">
         <v>3839028</v>
       </c>
@@ -6838,7 +6842,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="140" spans="1:13" ht="15.5" hidden="1">
+    <row r="140" spans="1:13" ht="15.5">
       <c r="A140" s="14">
         <v>1879172</v>
       </c>
@@ -6881,7 +6885,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="141" spans="1:13" ht="15.5" hidden="1">
+    <row r="141" spans="1:13" ht="15.5">
       <c r="A141" s="14">
         <v>1879042</v>
       </c>
@@ -6924,7 +6928,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="142" spans="1:13" ht="15.5" hidden="1">
+    <row r="142" spans="1:13" ht="15.5">
       <c r="A142" s="14">
         <v>3458038</v>
       </c>
@@ -6967,7 +6971,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="143" spans="1:13" ht="15.5" hidden="1">
+    <row r="143" spans="1:13" ht="15.5">
       <c r="A143" s="14">
         <v>1709041</v>
       </c>
@@ -7010,7 +7014,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="144" spans="1:13" ht="15.5" hidden="1">
+    <row r="144" spans="1:13" ht="15.5">
       <c r="A144" s="14">
         <v>2597033</v>
       </c>
@@ -7053,7 +7057,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="145" spans="1:13" ht="15.5" hidden="1">
+    <row r="145" spans="1:13" ht="15.5">
       <c r="A145" s="14">
         <v>1629041</v>
       </c>
@@ -7096,7 +7100,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="146" spans="1:13" ht="15.5" hidden="1">
+    <row r="146" spans="1:13" ht="15.5">
       <c r="A146" s="14">
         <v>1628041</v>
       </c>
@@ -7139,7 +7143,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="147" spans="1:13" ht="15.5" hidden="1">
+    <row r="147" spans="1:13" ht="15.5">
       <c r="A147" s="14">
         <v>1489033</v>
       </c>
@@ -7182,7 +7186,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="148" spans="1:13" ht="15.5" hidden="1">
+    <row r="148" spans="1:13" ht="15.5">
       <c r="A148" s="14">
         <v>1879041</v>
       </c>
@@ -7225,7 +7229,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="149" spans="1:13" ht="15.5" hidden="1">
+    <row r="149" spans="1:13" ht="15.5">
       <c r="A149" s="14">
         <v>2109013</v>
       </c>
@@ -7268,7 +7272,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="150" spans="1:13" ht="15.5" hidden="1">
+    <row r="150" spans="1:13" ht="15.5">
       <c r="A150" s="14">
         <v>1709033</v>
       </c>
@@ -7311,7 +7315,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="151" spans="1:13" ht="15.5" hidden="1">
+    <row r="151" spans="1:13" ht="15.5">
       <c r="A151" s="14">
         <v>3915041</v>
       </c>
@@ -7354,7 +7358,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="152" spans="1:13" ht="15.5" hidden="1">
+    <row r="152" spans="1:13" ht="15.5">
       <c r="A152" s="14">
         <v>1090005</v>
       </c>
@@ -7397,7 +7401,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="153" spans="1:13" ht="15.5" hidden="1">
+    <row r="153" spans="1:13" ht="15.5">
       <c r="A153" s="14">
         <v>3667418</v>
       </c>
@@ -7440,7 +7444,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="154" spans="1:13" ht="15.5" hidden="1">
+    <row r="154" spans="1:13" ht="15.5">
       <c r="A154" s="14">
         <v>1632033</v>
       </c>
@@ -7483,7 +7487,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="155" spans="1:13" ht="15.5" hidden="1">
+    <row r="155" spans="1:13" ht="15.5">
       <c r="A155" s="14">
         <v>1629033</v>
       </c>
@@ -7526,7 +7530,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="156" spans="1:13" ht="15.5" hidden="1">
+    <row r="156" spans="1:13" ht="15.5">
       <c r="A156" s="14">
         <v>1617041</v>
       </c>
@@ -7569,7 +7573,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="157" spans="1:13" ht="15.5" hidden="1">
+    <row r="157" spans="1:13" ht="15.5">
       <c r="A157" s="14">
         <v>1628033</v>
       </c>
@@ -7612,7 +7616,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="158" spans="1:13" ht="15.5" hidden="1">
+    <row r="158" spans="1:13" ht="15.5">
       <c r="A158" s="14">
         <v>1624033</v>
       </c>
@@ -7655,7 +7659,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="159" spans="1:13" ht="15.5" hidden="1">
+    <row r="159" spans="1:13" ht="15.5">
       <c r="A159" s="14">
         <v>1602033</v>
       </c>
@@ -7698,7 +7702,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="160" spans="1:13" ht="15.5" hidden="1">
+    <row r="160" spans="1:13" ht="15.5">
       <c r="A160" s="14">
         <v>2503033</v>
       </c>
@@ -7741,7 +7745,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="161" spans="1:13" ht="15.5" hidden="1">
+    <row r="161" spans="1:13" ht="15.5">
       <c r="A161" s="14">
         <v>1585041</v>
       </c>
@@ -7784,7 +7788,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="162" spans="1:13" ht="15.5" hidden="1">
+    <row r="162" spans="1:13" ht="15.5">
       <c r="A162" s="14">
         <v>1585041</v>
       </c>
@@ -7827,7 +7831,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="163" spans="1:13" ht="15.5" hidden="1">
+    <row r="163" spans="1:13" ht="15.5">
       <c r="A163" s="14">
         <v>3703041</v>
       </c>
@@ -7870,7 +7874,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="164" spans="1:13" ht="15.5" hidden="1">
+    <row r="164" spans="1:13" ht="15.5">
       <c r="A164" s="14">
         <v>3703041</v>
       </c>
@@ -7913,7 +7917,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="165" spans="1:13" ht="15.5" hidden="1">
+    <row r="165" spans="1:13" ht="15.5">
       <c r="A165" s="14">
         <v>1065033</v>
       </c>
@@ -7956,7 +7960,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="166" spans="1:13" ht="15.5" hidden="1">
+    <row r="166" spans="1:13" ht="15.5">
       <c r="A166" s="14">
         <v>2341041</v>
       </c>
@@ -7999,7 +8003,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="167" spans="1:13" ht="15.5" hidden="1">
+    <row r="167" spans="1:13" ht="15.5">
       <c r="A167" s="14">
         <v>1046172</v>
       </c>
@@ -8042,7 +8046,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="168" spans="1:13" ht="15.5" hidden="1">
+    <row r="168" spans="1:13" ht="15.5">
       <c r="A168" s="14">
         <v>1056100</v>
       </c>
@@ -8085,7 +8089,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="169" spans="1:13" ht="15.5" hidden="1">
+    <row r="169" spans="1:13" ht="15.5">
       <c r="A169" s="14">
         <v>2109048</v>
       </c>
@@ -8128,7 +8132,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="170" spans="1:13" ht="15.5" hidden="1">
+    <row r="170" spans="1:13" ht="15.5">
       <c r="A170" s="14">
         <v>1709112</v>
       </c>
@@ -8171,7 +8175,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="171" spans="1:13" ht="15.5" hidden="1">
+    <row r="171" spans="1:13" ht="15.5">
       <c r="A171" s="14">
         <v>1250013</v>
       </c>
@@ -8214,7 +8218,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="172" spans="1:13" ht="15.5" hidden="1">
+    <row r="172" spans="1:13" ht="15.5">
       <c r="A172" s="14">
         <v>3879041</v>
       </c>
@@ -8257,7 +8261,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="173" spans="1:13" ht="15.5" hidden="1">
+    <row r="173" spans="1:13" ht="15.5">
       <c r="A173" s="14">
         <v>3154041</v>
       </c>
@@ -8300,7 +8304,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="174" spans="1:13" ht="15.5" hidden="1">
+    <row r="174" spans="1:13" ht="15.5">
       <c r="A174" s="14">
         <v>1143013</v>
       </c>
@@ -8343,7 +8347,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="175" spans="1:13" ht="15.5" hidden="1">
+    <row r="175" spans="1:13" ht="15.5">
       <c r="A175" s="14">
         <v>1041172</v>
       </c>
@@ -8386,7 +8390,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="176" spans="1:13" ht="15.5" hidden="1">
+    <row r="176" spans="1:13" ht="15.5">
       <c r="A176" s="14">
         <v>3916041</v>
       </c>
@@ -8472,7 +8476,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="178" spans="1:13" ht="15.5" hidden="1">
+    <row r="178" spans="1:13" ht="15.5">
       <c r="A178" s="14">
         <v>2598013</v>
       </c>
@@ -8515,7 +8519,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="179" spans="1:13" ht="15.5" hidden="1">
+    <row r="179" spans="1:13" ht="15.5">
       <c r="A179" s="14">
         <v>1060172</v>
       </c>
@@ -8558,7 +8562,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="180" spans="1:13" ht="15.5" hidden="1">
+    <row r="180" spans="1:13" ht="15.5">
       <c r="A180" s="14">
         <v>1065091</v>
       </c>
@@ -8601,7 +8605,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="181" spans="1:13" ht="15.5" hidden="1">
+    <row r="181" spans="1:13" ht="15.5">
       <c r="A181" s="14">
         <v>1065091</v>
       </c>
@@ -8644,7 +8648,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="182" spans="1:13" ht="15.5" hidden="1">
+    <row r="182" spans="1:13" ht="15.5">
       <c r="A182" s="14">
         <v>3891482</v>
       </c>
@@ -8687,7 +8691,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="183" spans="1:13" ht="15.5" hidden="1">
+    <row r="183" spans="1:13" ht="15.5">
       <c r="A183" s="14">
         <v>1873172</v>
       </c>
@@ -8730,7 +8734,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="184" spans="1:13" ht="15.5" hidden="1">
+    <row r="184" spans="1:13" ht="15.5">
       <c r="A184" s="14">
         <v>1933621</v>
       </c>
@@ -8773,7 +8777,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="185" spans="1:13" ht="15.5" hidden="1">
+    <row r="185" spans="1:13" ht="15.5">
       <c r="A185" s="14">
         <v>3715041</v>
       </c>
@@ -8816,7 +8820,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="186" spans="1:13" ht="15.5" hidden="1">
+    <row r="186" spans="1:13" ht="15.5">
       <c r="A186" s="14">
         <v>1599211</v>
       </c>
@@ -8859,7 +8863,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="187" spans="1:13" ht="15.5" hidden="1">
+    <row r="187" spans="1:13" ht="15.5">
       <c r="A187" s="14">
         <v>1709211</v>
       </c>
@@ -8902,7 +8906,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="188" spans="1:13" ht="15.5" hidden="1">
+    <row r="188" spans="1:13" ht="15.5">
       <c r="A188" s="14">
         <v>1496224</v>
       </c>
@@ -8945,7 +8949,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="189" spans="1:13" ht="15.5" hidden="1">
+    <row r="189" spans="1:13" ht="15.5">
       <c r="A189" s="14">
         <v>1065211</v>
       </c>
@@ -8988,7 +8992,7 @@
         <v>+</v>
       </c>
     </row>
-    <row r="190" spans="1:13" ht="15.5" hidden="1">
+    <row r="190" spans="1:13" ht="15.5">
       <c r="A190" s="14">
         <v>1363130</v>
       </c>
@@ -9032,13 +9036,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A8:M190" xr:uid="{F88453A7-FECA-4927-826D-F01BE31EC038}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="BUD LIGHT LIME TIME"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A8:M190" xr:uid="{F88453A7-FECA-4927-826D-F01BE31EC038}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A9:K190">
     <sortCondition ref="C9:C190"/>
     <sortCondition ref="D9:D190"/>
@@ -9064,27 +9062,22 @@
 </worksheet>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1F29A87-C711-452F-84A0-6436361D6E8E}">
+  <dimension ref="F2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="2" spans="6:6">
+      <c r="F2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4d19c67b-01ac-4d4b-a843-fb81d321b596">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="6dca17fb-ac11-4cf8-b45b-b93bf268ff03" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003BD24DCF8EBA2A459A3767B75ECBC810" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="14ba1abd425e7d287f53e65cd7fdc17f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4d19c67b-01ac-4d4b-a843-fb81d321b596" xmlns:ns3="6dca17fb-ac11-4cf8-b45b-b93bf268ff03" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f877f0b356da1ae16043b73a66e5efc3" ns2:_="" ns3:_="">
     <xsd:import namespace="4d19c67b-01ac-4d4b-a843-fb81d321b596"/>
@@ -9339,32 +9332,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B6DF62D-6E20-4488-8172-8E2FED293569}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E560CAD-3D0D-4622-8ACC-0E2F5560BCED}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="6dca17fb-ac11-4cf8-b45b-b93bf268ff03"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4d19c67b-01ac-4d4b-a843-fb81d321b596"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4d19c67b-01ac-4d4b-a843-fb81d321b596">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="6dca17fb-ac11-4cf8-b45b-b93bf268ff03" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{663EA9A2-C52A-4722-944D-0B4351AA8E9D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9381,4 +9369,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B6DF62D-6E20-4488-8172-8E2FED293569}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E560CAD-3D0D-4622-8ACC-0E2F5560BCED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="6dca17fb-ac11-4cf8-b45b-b93bf268ff03"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4d19c67b-01ac-4d4b-a843-fb81d321b596"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>